<commit_message>
Mise à jour : ajout de la javadoc.
</commit_message>
<xml_diff>
--- a/BaseDeDonnee.xlsx
+++ b/BaseDeDonnee.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="63">
   <si>
     <t>Jours</t>
   </si>
@@ -283,7 +283,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5">

</xml_diff>